<commit_message>
task 6 and 7 added
</commit_message>
<xml_diff>
--- a/data/raw_data.xlsx
+++ b/data/raw_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Private\555 sha\P\pandas-data-cleaning-project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E09E3F0-EBDF-448B-8FFD-E64EE5FD5CF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A009BC63-54EA-4ADC-8897-D4D85B990769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6652,7 +6652,7 @@
         <v>6500</v>
       </c>
       <c r="F17" t="s">
-        <v>959</v>
+        <v>1007</v>
       </c>
       <c r="G17" t="s">
         <v>991</v>

</xml_diff>